<commit_message>
Remove internal editing-history annotations from Supplementary Table S5 Notes
Per author decision (reviewed and agreed by all authors and the external
reviewer), the bracketed process annotations left in the Notes columns of
both the QUIN_in_vitro and SYRCLE_in_vivo sheets -- "[Armonizacion
2026-10-18: ...]" and "[CORREGIDO 2026-10-19/2026-10-20: ...]" -- are
removed. These were internal working notes documenting a two-step
editing history (an earlier harmonization pass, followed by a correction
pass whose stated premise about SYRCLE's default convention was itself
incorrect); the underlying risk-of-bias ratings corrected in the previous
commit (D8/D9/D10 recoded to Unclear where unsupported) are unaffected
and remain in place. The Supplementary Table S5 caveat cell (SYRCLE_in_vivo
A2) is simplified accordingly, keeping the substantive SYRCLE Unclear-vs-Yes
methodology disclosure and dropping the now-removed mention of the
2026-10-19 annotation.
</commit_message>
<xml_diff>
--- a/supplementary/Supplementary_Table_S5_Risk_of_Bias_QUIN_SYRCLE.xlsx
+++ b/supplementary/Supplementary_Table_S5_Risk_of_Bias_QUIN_SYRCLE.xlsx
@@ -524,6 +524,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -709,7 +710,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Aims, controls (solid-core vs hollow fiber), fabrication protocol, and stats (GraphPad, ANOVA/Tukey) are clearly reported, but sample size is explicitly stated as chosen 'for feasibility' rather than power-justified, and operator identity, assessor blinding/inter-rater reliability, and randomization of in vitro group allocation are never mentioned. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Aims, controls (solid-core vs hollow fiber), fabrication protocol, and stats (GraphPad, ANOVA/Tukey) are clearly reported, but sample size is explicitly stated as chosen 'for feasibility' rather than power-justified, and operator identity, assessor blinding/inter-rater reliability, and randomization of in vitro group allocation are never mentioned.</t>
         </is>
       </c>
       <c r="Q4" t="n">
@@ -799,7 +800,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Very detailed, replicable material/hydrogel fabrication and characterization methods with clear composition-based comparison groups and a well-specified statistics section (one-/two-way ANOVA, Tukey/Dunnett post hoc), but replicate numbers (n=3) are not power-justified, and operator identity, outcome-assessor blinding/inter-rater reliability, and randomization of cell/scaffold group allocation are not reported. Purely in vitro (cell line iMSC#3); no animal component. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Very detailed, replicable material/hydrogel fabrication and characterization methods with clear composition-based comparison groups and a well-specified statistics section (one-/two-way ANOVA, Tukey/Dunnett post hoc), but replicate numbers (n=3) are not power-justified, and operator identity, outcome-assessor blinding/inter-rater reliability, and randomization of cell/scaffold group allocation are not reported. Purely in vitro (cell line iMSC#3); no animal component.</t>
         </is>
       </c>
       <c r="Q5" t="n">
@@ -889,7 +890,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Clear aims, well-described scaffold groups (single-layer PCL, tri-layer PVA/PCL/PVA, core-shell) and controls, detailed electrospinning/testing protocols, and an explicit statistics section (SPSS one-way ANOVA, p&lt;0.05), but sample sizes (n=3-6) lack power justification and there is no mention of operator identity, randomization, or blinding at any stage. Only HEK-293 cell culture used; no animal work (in vitro only). [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Clear aims, well-described scaffold groups (single-layer PCL, tri-layer PVA/PCL/PVA, core-shell) and controls, detailed electrospinning/testing protocols, and an explicit statistics section (SPSS one-way ANOVA, p&lt;0.05), but sample sizes (n=3-6) lack power justification and there is no mention of operator identity, randomization, or blinding at any stage. Only HEK-293 cell culture used; no animal work (in vitro only).</t>
         </is>
       </c>
       <c r="Q6" t="n">
@@ -979,7 +980,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Aims, scaffold groups (PCL, PCL/HA, PCL/HA/GO@SPION) and comparisons are clear, methodology (RT-PCR, ALP, IHC, alizarin red) is detailed with an explicit statistics section (one-way ANOVA, Tukey post hoc), but sample size is not power-justified, and operator/assessor identity, randomization of well/sample allocation, and blinding are never described. Purely in vitro (AdMSCs); no in vivo work despite the future-work framing. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Aims, scaffold groups (PCL, PCL/HA, PCL/HA/GO@SPION) and comparisons are clear, methodology (RT-PCR, ALP, IHC, alizarin red) is detailed with an explicit statistics section (one-way ANOVA, Tukey post hoc), but sample size is not power-justified, and operator/assessor identity, randomization of well/sample allocation, and blinding are never described. Purely in vitro (AdMSCs); no in vivo work despite the future-work framing.</t>
         </is>
       </c>
       <c r="Q7" t="n">
@@ -1069,7 +1070,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Nine scaffold formulations are clearly tabulated with comparison groups, fabrication is well described, and statistics are explicit (Minitab, one-way ANOVA + Tukey, paired t-test for viability), but sample size (n=3-6) is not power-justified and operator identity, randomization, assessor blinding/inter-rater reliability are not reported. In vitro only (C2C12 cells, MTT/degradation/swelling); no animal work. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Nine scaffold formulations are clearly tabulated with comparison groups, fabrication is well described, and statistics are explicit (Minitab, one-way ANOVA + Tukey, paired t-test for viability), but sample size (n=3-6) is not power-justified and operator identity, randomization, assessor blinding/inter-rater reliability are not reported. In vitro only (C2C12 cells, MTT/degradation/swelling); no animal work.</t>
         </is>
       </c>
       <c r="Q8" t="n">
@@ -1159,7 +1160,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Short (4-page) letter with clear scaffold groups (Control, PC, PCFC, OPCFC⊥/∥) and standardized characterization equipment, results shown with error bars and significance markers (n=4), but no dedicated statistics section names the actual test/software used, sample size is not justified, and operator identity, randomization, and blinding are not addressed anywhere. In vitro only (MC3T3-E1 cells); authors explicitly frame in vivo work as future research. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Short (4-page) letter with clear scaffold groups (Control, PC, PCFC, OPCFC⊥/∥) and standardized characterization equipment, results shown with error bars and significance markers (n=4), but no dedicated statistics section names the actual test/software used, sample size is not justified, and operator identity, randomization, and blinding are not addressed anywhere. In vitro only (MC3T3-E1 cells); authors explicitly frame in vivo work as future research.</t>
         </is>
       </c>
       <c r="Q9" t="n">
@@ -1249,7 +1250,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>In vitro angiogenesis (HUVEC tube formation) and cell-alignment (3T3) experiments have clear control groups and standardized imaging/quantification (n=3), but no methods paragraph specifies the statistical test/software used (only significance asterisks appear in figure legends), sample size is not power-justified, and operator identity, randomization, and blinding are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro angiogenesis (HUVEC tube formation) and cell-alignment (3T3) experiments have clear control groups and standardized imaging/quantification (n=3), but no methods paragraph specifies the statistical test/software used (only significance asterisks appear in figure legends), sample size is not power-justified, and operator identity, randomization, and blinding are not reported.</t>
         </is>
       </c>
       <c r="Q10" t="n">
@@ -1339,7 +1340,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>In vitro cytotoxicity, hemolysis and degradation assays use clear scaffold comparison groups and an explicit statistics method (Origin Pro, ANOVA, p&lt;0.05), but sample size is not power-justified, and operator identity, randomization of sample/well allocation, and assessor blinding are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro cytotoxicity, hemolysis and degradation assays use clear scaffold comparison groups and an explicit statistics method (Origin Pro, ANOVA, p&lt;0.05), but sample size is not power-justified, and operator identity, randomization of sample/well allocation, and assessor blinding are not reported.</t>
         </is>
       </c>
       <c r="Q11" t="n">
@@ -1429,7 +1430,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>In vitro cytocompatibility, scratch and transwell assays have multiple clear comparison groups (TPU, TPU/CS, TPU/CS@ZnO) and an explicit statistics method (two-tailed t-test), but sample sizes are not power-justified and operator identity, randomization, and blinding are not addressed. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro cytocompatibility, scratch and transwell assays have multiple clear comparison groups (TPU, TPU/CS, TPU/CS@ZnO) and an explicit statistics method (two-tailed t-test), but sample sizes are not power-justified and operator identity, randomization, and blinding are not addressed.</t>
         </is>
       </c>
       <c r="Q12" t="n">
@@ -1519,7 +1520,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>In vitro hBMSC/HUVEC transwell-migration and tubule-formation assays have clear peptide-based comparison groups (Control, BMHP, VP, BMHP+VP) and an explicit statistics section (one-way ANOVA, LSD post hoc), but sample size is not power-justified and operator identity, randomization, and blinding are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro hBMSC/HUVEC transwell-migration and tubule-formation assays have clear peptide-based comparison groups (Control, BMHP, VP, BMHP+VP) and an explicit statistics section (one-way ANOVA, LSD post hoc), but sample size is not power-justified and operator identity, randomization, and blinding are not reported.</t>
         </is>
       </c>
       <c r="Q13" t="n">
@@ -1699,7 +1700,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Clear aims, control/comparator groups, detailed synthesis chemistry and appropriate statistics (ANOVA, GraphPad Prism) are reported, but no sample-size justification, no randomization of replicates, no operator or assessor detail, and no blinding anywhere in the study. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Clear aims, control/comparator groups, detailed synthesis chemistry and appropriate statistics (ANOVA, GraphPad Prism) are reported, but no sample-size justification, no randomization of replicates, no operator or assessor detail, and no blinding anywhere in the study.</t>
         </is>
       </c>
       <c r="Q15" t="n">
@@ -1789,7 +1790,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>The in vitro component is a scaffold release/degradation material study (no cultured cells): clear aims, a blank-CCS comparator and standardized ICP-MS/gravimetric measurement with proper statistics are used, but sample-size justification, randomization, operator/assessor detail and blinding are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>The in vitro component is a scaffold release/degradation material study (no cultured cells): clear aims, a blank-CCS comparator and standardized ICP-MS/gravimetric measurement with proper statistics are used, but sample-size justification, randomization, operator/assessor detail and blinding are not reported.</t>
         </is>
       </c>
       <c r="Q16" t="n">
@@ -1879,7 +1880,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>BMSC in vitro assays have clear aims, PLA/DAPLA comparator groups, detailed fabrication protocols, standardized assays (CCK-8, ALP, qPCR) and SPSS-based statistics, but no sample-size justification, randomization, operator/assessor detail or blinding are reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>BMSC in vitro assays have clear aims, PLA/DAPLA comparator groups, detailed fabrication protocols, standardized assays (CCK-8, ALP, qPCR) and SPSS-based statistics, but no sample-size justification, randomization, operator/assessor detail or blinding are reported.</t>
         </is>
       </c>
       <c r="Q17" t="n">
@@ -1969,7 +1970,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>BMSC/MC3T3-E1 in vitro assays are clearly described with Blank/CS/CS-SF/CS-SF@SrAlg comparator groups, detailed methods and one-way ANOVA with Tukey's test, but sample size is not justified and randomization, operator/assessor detail and blinding are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>BMSC/MC3T3-E1 in vitro assays are clearly described with Blank/CS/CS-SF/CS-SF@SrAlg comparator groups, detailed methods and one-way ANOVA with Tukey's test, but sample size is not justified and randomization, operator/assessor detail and blinding are not reported.</t>
         </is>
       </c>
       <c r="Q18" t="n">
@@ -2059,7 +2060,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>BV2/PC12/HUVEC/L929 cell-culture experiments have clear aims, TCP/LPS controls, detailed WBPU synthesis and ANOVA-based statistics with exact p-values, but no sample-size justification, randomization, operator/assessor detail or blinding are reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>BV2/PC12/HUVEC/L929 cell-culture experiments have clear aims, TCP/LPS controls, detailed WBPU synthesis and ANOVA-based statistics with exact p-values, but no sample-size justification, randomization, operator/assessor detail or blinding are reported.</t>
         </is>
       </c>
       <c r="Q19" t="n">
@@ -2149,7 +2150,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Materials-focused polyHIPE paper; the single cell-growth experiment (MSC/HUVEC on constructs, with cell passage numbers reported and a PLLA/PLGA salt-leached reference scaffold as comparator) is reported qualitatively via Live/Dead confocal images without quantified viability values, a named statistical test, sample-size justification, randomization or blinding. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Materials-focused polyHIPE paper; the single cell-growth experiment (MSC/HUVEC on constructs, with cell passage numbers reported and a PLLA/PLGA salt-leached reference scaffold as comparator) is reported qualitatively via Live/Dead confocal images without quantified viability values, a named statistical test, sample-size justification, randomization or blinding.</t>
         </is>
       </c>
       <c r="Q20" t="n">
@@ -2239,7 +2240,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>MG-63 cell assays have clear aims, PnH/PnH-A/PnH-A-G comparator groups, detailed aminolysis/gelatin-coating protocols and ANOVA-based statistics (triplicate testing), but no sample-size justification, randomization, operator/assessor detail or blinding are reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MG-63 cell assays have clear aims, PnH/PnH-A/PnH-A-G comparator groups, detailed aminolysis/gelatin-coating protocols and ANOVA-based statistics (triplicate testing), but no sample-size justification, randomization, operator/assessor detail or blinding are reported.</t>
         </is>
       </c>
       <c r="Q21" t="n">
@@ -2329,7 +2330,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>MC3T3-E1 cell assays have clear aims, a 0% ZnO/CS control plus dose-graded comparator groups, detailed fabrication and ANOVA statistics, but no sample-size justification, randomization, operator/assessor detail or blinding are reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MC3T3-E1 cell assays have clear aims, a 0% ZnO/CS control plus dose-graded comparator groups, detailed fabrication and ANOVA statistics, but no sample-size justification, randomization, operator/assessor detail or blinding are reported.</t>
         </is>
       </c>
       <c r="Q22" t="n">
@@ -2419,7 +2420,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>C2C12 cell-viability (WST-1) and bacterial-inhibition (E. coli/H. pylori CFU) assays have clear aims, untreated-control comparisons and detailed ALD/synthesis protocols with triplicate testing, but no sample-size justification, randomization, operator/assessor detail or blinding were found, and the statistical treatment/quantitative results of the biological assays were not confirmed in the pages reviewed. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>C2C12 cell-viability (WST-1) and bacterial-inhibition (E. coli/H. pylori CFU) assays have clear aims, untreated-control comparisons and detailed ALD/synthesis protocols with triplicate testing, but no sample-size justification, randomization, operator/assessor detail or blinding were found, and the statistical treatment/quantitative results of the biological assays were not confirmed in the pages reviewed.</t>
         </is>
       </c>
       <c r="Q23" t="n">
@@ -2509,7 +2510,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>Clear aims, detailed fabrication/culture protocols, defined control groups (static culture, TCP), standardized outcome measures and ANOVA/Tukey statistics with mean±SD reporting. No sample-size justification beyond a bare n=3, and no randomization, operator, or blinding details are reported anywhere. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Clear aims, detailed fabrication/culture protocols, defined control groups (static culture, TCP), standardized outcome measures and ANOVA/Tukey statistics with mean±SD reporting. No sample-size justification beyond a bare n=3, and no randomization, operator, or blinding details are reported anywhere.</t>
         </is>
       </c>
       <c r="Q24" t="n">
@@ -2599,7 +2600,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>MTT cytotoxicity and antibacterial assays follow standard protocols (ISO 10993-5, agar diffusion) with a stated cell line/source, but no statistical test (e.g., ANOVA/t-test) or variance measure is reported for the cytotoxicity data (bar graph has no error bars), and no sample-size justification, randomization, operator detail, or blinding is described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MTT cytotoxicity and antibacterial assays follow standard protocols (ISO 10993-5, agar diffusion) with a stated cell line/source, but no statistical test (e.g., ANOVA/t-test) or variance measure is reported for the cytotoxicity data (bar graph has no error bars), and no sample-size justification, randomization, operator detail, or blinding is described.</t>
         </is>
       </c>
       <c r="Q25" t="n">
@@ -2689,7 +2690,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>In vitro chondrocyte biocompatibility (live/dead, CCK-8) is well described with a clear control (CM sponge) and one-way ANOVA statistics with error bars, but sample size is only a bare n (3-4) with no justification, and no randomization, operator, or blinding details are given. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro chondrocyte biocompatibility (live/dead, CCK-8) is well described with a clear control (CM sponge) and one-way ANOVA statistics with error bars, but sample size is only a bare n (3-4) with no justification, and no randomization, operator, or blinding details are given.</t>
         </is>
       </c>
       <c r="Q26" t="n">
@@ -2869,7 +2870,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>MG-63 in vitro assays (MTT, CCK-8, ALP, alizarin red) are clearly described with a no-scaffold control and paired t-test/ANOVA statistics, but sample size is only stated as 'three replicates' without justification, and no randomization, operator, or blinding details are reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MG-63 in vitro assays (MTT, CCK-8, ALP, alizarin red) are clearly described with a no-scaffold control and paired t-test/ANOVA statistics, but sample size is only stated as 'three replicates' without justification, and no randomization, operator, or blinding details are reported.</t>
         </is>
       </c>
       <c r="Q28" t="n">
@@ -2959,7 +2960,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>Well-controlled 2D/transwell osteoblast experiments (NG vs HG, PC/PCG/PCMG coatings) with a defined cell line, standardized assays (live/dead, ALP, RT-qPCR) and ANOVA/Tukey-Kramer statistics with n=3 triplicates, but no formal sample-size justification and no randomization or blinding of culture handling/assessment described. Authors explicitly flag in vivo evaluation as future work, confirming no animal component here. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Well-controlled 2D/transwell osteoblast experiments (NG vs HG, PC/PCG/PCMG coatings) with a defined cell line, standardized assays (live/dead, ALP, RT-qPCR) and ANOVA/Tukey-Kramer statistics with n=3 triplicates, but no formal sample-size justification and no randomization or blinding of culture handling/assessment described. Authors explicitly flag in vivo evaluation as future work, confirming no animal component here.</t>
         </is>
       </c>
       <c r="Q29" t="n">
@@ -3229,7 +3230,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>In vitro BMSC/RAEC dynamic-culture experiments (live/dead, CCK-8, ALP, ARS, CD31/Runx2 staining) are clearly described with a static-culture control and one-way ANOVA/LSD statistics (n≥3), but sample size is only a bare n with no justification, and no randomization, operator, or blinding details are reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro BMSC/RAEC dynamic-culture experiments (live/dead, CCK-8, ALP, ARS, CD31/Runx2 staining) are clearly described with a static-culture control and one-way ANOVA/LSD statistics (n≥3), but sample size is only a bare n with no justification, and no randomization, operator, or blinding details are reported.</t>
         </is>
       </c>
       <c r="Q32" t="n">
@@ -3319,7 +3320,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>MG-63 MTT/ALP/attachment assays across three scaffold compositions are clearly described with mean±SD reporting and a stated significance threshold (P≤0.05), but the specific statistical test (e.g., ANOVA) is not named, sample size for the cell assays is not explicitly justified, and no randomization, operator, or blinding details are reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MG-63 MTT/ALP/attachment assays across three scaffold compositions are clearly described with mean±SD reporting and a stated significance threshold (P≤0.05), but the specific statistical test (e.g., ANOVA) is not named, sample size for the cell assays is not explicitly justified, and no randomization, operator, or blinding details are reported.</t>
         </is>
       </c>
       <c r="Q33" t="n">
@@ -3409,7 +3410,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>WI-38 cytotoxicity (ISO 10993-12/MTT) and antibacterial assays are clearly described with a blank/control scaffold and Student's t-test statistics (n=3, mean±SD) reported explicitly, but sample size is only a bare n with no formal justification, and no randomization, operator, or blinding details are given. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>WI-38 cytotoxicity (ISO 10993-12/MTT) and antibacterial assays are clearly described with a blank/control scaffold and Student's t-test statistics (n=3, mean±SD) reported explicitly, but sample size is only a bare n with no formal justification, and no randomization, operator, or blinding details are given.</t>
         </is>
       </c>
       <c r="Q34" t="n">
@@ -3589,7 +3590,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Very detailed fabrication/assay methods and standardized outcome measures with clear statistics (ANOVA/t-tests, GraphPad Prism), but no sample-size justification, no operator details, no randomization or blinding of cell-based assays reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Very detailed fabrication/assay methods and standardized outcome measures with clear statistics (ANOVA/t-tests, GraphPad Prism), but no sample-size justification, no operator details, no randomization or blinding of cell-based assays reported.</t>
         </is>
       </c>
       <c r="Q36" t="n">
@@ -3679,7 +3680,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Unusually rigorous statistical framework (mixed-effects models, plate-level random effects, Cohen's d, one-sample t-tests vs ISO threshold, minimum 4 replicates justified by regulatory design), but operator identity/training, randomization of sample allocation, and blinding of outcome assessment are not reported. [Correccion Q11 tras revision del texto completo, 2026-10-18: No se identifica el nombre del software estadistico (solo ANOVA, Tukey HSD, Cohen's d, modelo mixto); bajo el criterio estricto acordado (Q11 requiere software nombrado), queda Unclear, no Yes.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Unusually rigorous statistical framework (mixed-effects models, plate-level random effects, Cohen's d, one-sample t-tests vs ISO threshold, minimum 4 replicates justified by regulatory design), but operator identity/training, randomization of sample allocation, and blinding of outcome assessment are not reported. [Correccion Q11 tras revision del texto completo, 2026-10-18: No se identifica el nombre del software estadistico (solo ANOVA, Tukey HSD, Cohen's d, modelo mixto); bajo el criterio estricto acordado (Q11 requiere software nombrado), queda Unclear, no Yes.]</t>
         </is>
       </c>
       <c r="Q37" t="n">
@@ -3769,7 +3770,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>CCK-8 cytotoxicity and hemolysis assays (each run in triplicate) are described but no formal statistical test (ANOVA/t-test) is ever named; no operator, randomization, or blinding details given. Note: a section titled 'In Vitro and in Vivo Biocompatibility' is misleading -- it only covers in vitro CCK-8 and ex vivo rabbit-blood hemolysis; the conclusion explicitly states true in vivo degradation studies are left to 'future work', confirming no live-animal experiments were performed. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>CCK-8 cytotoxicity and hemolysis assays (each run in triplicate) are described but no formal statistical test (ANOVA/t-test) is ever named; no operator, randomization, or blinding details given. Note: a section titled 'In Vitro and in Vivo Biocompatibility' is misleading -- it only covers in vitro CCK-8 and ex vivo rabbit-blood hemolysis; the conclusion explicitly states true in vivo degradation studies are left to 'future work', confirming no live-animal experiments were performed.</t>
         </is>
       </c>
       <c r="Q38" t="n">
@@ -3859,7 +3860,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>MTS assay at 4 timepoints described only qualitatively (no replicate number, no error bars/variance, no named statistical test); paper explicitly states no animal/human-participant experiments were performed. Fabrication methodology otherwise well described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MTS assay at 4 timepoints described only qualitatively (no replicate number, no error bars/variance, no named statistical test); paper explicitly states no animal/human-participant experiments were performed. Fabrication methodology otherwise well described.</t>
         </is>
       </c>
       <c r="Q39" t="n">
@@ -3949,7 +3950,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Comprehensive characterization and MTT viability assays with clear statistics (one-way ANOVA, Tukey post hoc, SPSS) and n&gt;=3, but no sample-size justification, operator details, randomization, or blinding are reported. Authors explicitly note future work will include in vivo evaluation, confirming none was performed here. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Comprehensive characterization and MTT viability assays with clear statistics (one-way ANOVA, Tukey post hoc, SPSS) and n&gt;=3, but no sample-size justification, operator details, randomization, or blinding are reported. Authors explicitly note future work will include in vivo evaluation, confirming none was performed here.</t>
         </is>
       </c>
       <c r="Q40" t="n">
@@ -4039,7 +4040,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>Rigorous statistics (Shapiro-Wilk, Levene, one-way ANOVA with Tukey post hoc) and detailed hADSC culture/osteogenic-differentiation protocols, but no sample-size justification, operator/training details, randomization, or blinding reported. Abstract explicitly notes only feasibility for 'future in vivo research' was evaluated -- confirming no animal work in this paper. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Rigorous statistics (Shapiro-Wilk, Levene, one-way ANOVA with Tukey post hoc) and detailed hADSC culture/osteogenic-differentiation protocols, but no sample-size justification, operator/training details, randomization, or blinding reported. Abstract explicitly notes only feasibility for 'future in vivo research' was evaluated -- confirming no animal work in this paper.</t>
         </is>
       </c>
       <c r="Q41" t="n">
@@ -4129,7 +4130,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>AlamarBlue cell-proliferation assay compares rADSCs on PCL, dPCL and dPCL/HA scaffolds with bar-graph error bars, but no statistical test (ANOVA/t-test) is named anywhere in the manuscript, and no sample-size justification, operator, or blinding details are given. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>AlamarBlue cell-proliferation assay compares rADSCs on PCL, dPCL and dPCL/HA scaffolds with bar-graph error bars, but no statistical test (ANOVA/t-test) is named anywhere in the manuscript, and no sample-size justification, operator, or blinding details are given.</t>
         </is>
       </c>
       <c r="Q42" t="n">
@@ -4219,7 +4220,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>Very detailed extraction/fabrication methods and clear statistics (one-way ANOVA, 95% CI, n&gt;=3), human nail donation described as following approved SOPs, but no formal sample-size justification, no operator/training detail, no randomization of scaffold-to-well allocation, and no blinding of manual trypan-blue cell counts. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Very detailed extraction/fabrication methods and clear statistics (one-way ANOVA, 95% CI, n&gt;=3), human nail donation described as following approved SOPs, but no formal sample-size justification, no operator/training detail, no randomization of scaffold-to-well allocation, and no blinding of manual trypan-blue cell counts.</t>
         </is>
       </c>
       <c r="Q43" t="n">
@@ -4309,7 +4310,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>MTT assay on MG63 cells per ISO-10993 with one-way ANOVA (p&lt;0.05) and mean+/-SD reporting, and bioactivity assessed via SBF immersion (not animal), but no sample-size justification, operator/training detail, randomization, or blinding reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MTT assay on MG63 cells per ISO-10993 with one-way ANOVA (p&lt;0.05) and mean+/-SD reporting, and bioactivity assessed via SBF immersion (not animal), but no sample-size justification, operator/training detail, randomization, or blinding reported.</t>
         </is>
       </c>
       <c r="Q44" t="n">
@@ -4579,7 +4580,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Clear aims, methods, controls (2D mat/dropcast/PTP), stated replicate number (n=6) and ANOVA/Tukey statistics with exact p-values. No mention of operator details, randomization of well allocation, assessor blinding, or inter-rater reliability, which are the main gaps. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "n = 6" sin ninguna justificacion numerica o estadistica de por que se elige ese tamano; no hay calculo de poder ni referencia a un estandar. Bajo el criterio estricto (Q2 requiere justificacion real, no solo declarar el numero de replicas), queda Unclear, no Yes.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Clear aims, methods, controls (2D mat/dropcast/PTP), stated replicate number (n=6) and ANOVA/Tukey statistics with exact p-values. No mention of operator details, randomization of well allocation, assessor blinding, or inter-rater reliability, which are the main gaps. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "n = 6" sin ninguna justificacion numerica o estadistica de por que se elige ese tamano; no hay calculo de poder ni referencia a un estandar. Bajo el criterio estricto (Q2 requiere justificacion real, no solo declarar el numero de replicas), queda Unclear, no Yes.]</t>
         </is>
       </c>
       <c r="Q47" t="n">
@@ -4669,7 +4670,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>The file under W03 is a different, much shorter paper (Materials Letters short communication) on Mg/Sr-modified hydroxyapatite whisker scaffolds, not the expected Zhu et al. cellulose-nanocrystal/HA/PVA paper. Methods are minimal: no cell source/passage details, no stated replicate numbers for CCK-8/ALP, no statistical test named anywhere, and ALP results shown only as unquantified images. | RECOVERY NOTE: This is the TRUE W07 study content, found inside a file that was incorrectly named "W03.pdf". The W03.pdf filename does not contain the real W03 study (Zhu et al., cellulose nanocrystal/HA/PVA), which is still missing. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>The file under W03 is a different, much shorter paper (Materials Letters short communication) on Mg/Sr-modified hydroxyapatite whisker scaffolds, not the expected Zhu et al. cellulose-nanocrystal/HA/PVA paper. Methods are minimal: no cell source/passage details, no stated replicate numbers for CCK-8/ALP, no statistical test named anywhere, and ALP results shown only as unquantified images. | RECOVERY NOTE: This is the TRUE W07 study content, found inside a file that was incorrectly named "W03.pdf". The W03.pdf filename does not contain the real W03 study (Zhu et al., cellulose nanocrystal/HA/PVA), which is still missing.</t>
         </is>
       </c>
       <c r="Q48" t="n">
@@ -4849,7 +4850,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>In vitro portion (BMSC osteoblast induction, SBF degradation, alamarBlue proliferation) has clear aims, groups (E0-E4), triplicate-combined statistics (t-test/ANOVA), and adequately presented results. No operator, randomization, assessor, or blinding details given. [Correccion Q2 tras revision del texto completo, 2026-10-18: El calculo de tamano de muestra con el programa PSTM se aplica explicitamente "the sample size of the animal experiment" (SYRCLE/in vivo), no a la porcion in vitro, que solo declara "3 individual experiments... combined for statistical analysis" sin justificacion propia. Para QUIN (in vitro) queda Unclear, no Yes.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro portion (BMSC osteoblast induction, SBF degradation, alamarBlue proliferation) has clear aims, groups (E0-E4), triplicate-combined statistics (t-test/ANOVA), and adequately presented results. No operator, randomization, assessor, or blinding details given. [Correccion Q2 tras revision del texto completo, 2026-10-18: El calculo de tamano de muestra con el programa PSTM se aplica explicitamente "the sample size of the animal experiment" (SYRCLE/in vivo), no a la porcion in vitro, que solo declara "3 individual experiments... combined for statistical analysis" sin justificacion propia. Para QUIN (in vitro) queda Unclear, no Yes.]</t>
         </is>
       </c>
       <c r="Q50" t="n">
@@ -4939,7 +4940,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>Short-communication format (Materials Letters). Material/pore-size and nHAP-content comparison groups clearly defined and results shown with error bars, but sample size/replicate numbers for compression and cytotoxicity/adhesion tests, the specific cytotoxicity assay protocol, and the statistical test used are not clearly stated in the main text (may be in unread supplementary data); no operator, randomization, assessor, or blinding details given. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Short-communication format (Materials Letters). Material/pore-size and nHAP-content comparison groups clearly defined and results shown with error bars, but sample size/replicate numbers for compression and cytotoxicity/adhesion tests, the specific cytotoxicity assay protocol, and the statistical test used are not clearly stated in the main text (may be in unread supplementary data); no operator, randomization, assessor, or blinding details given.</t>
         </is>
       </c>
       <c r="Q51" t="n">
@@ -5119,7 +5120,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Well-reported core-shell electrospun scaffold study: clear aims, triplicate analyses stated ('all experimental analyses were conducted in triplicate'), defined comparison groups (0E/1E/3E/5E), standardized assays (MTT, qRT-PCR with defined primers) and two-way ANOVA with GraphPad Prism. No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Declara "triplicate to ensure statistical robustness" y n=3 segun ASTM D882 para el ensayo mecanico, pero no hay justificacion estadistica real (calculo de poder o referencia) de por que ese numero es adecuado; el estandar ASTM especifica el procedimiento, no justifica el tamano de muestra biologico. Queda Unclear, no Yes.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Well-reported core-shell electrospun scaffold study: clear aims, triplicate analyses stated ('all experimental analyses were conducted in triplicate'), defined comparison groups (0E/1E/3E/5E), standardized assays (MTT, qRT-PCR with defined primers) and two-way ANOVA with GraphPad Prism. No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Declara "triplicate to ensure statistical robustness" y n=3 segun ASTM D882 para el ensayo mecanico, pero no hay justificacion estadistica real (calculo de poder o referencia) de por que ese numero es adecuado; el estandar ASTM especifica el procedimiento, no justifica el tamano de muestra biologico. Queda Unclear, no Yes.]</t>
         </is>
       </c>
       <c r="Q53" t="n">
@@ -5209,7 +5210,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>In vitro portion (MC3T3-E1 cell viability/adhesion on HG/XG/WG chitosan gels) is well described: aims clear, 'all experiments repeated at least three times', defined comparison groups and controls, standardized CCK-8/live-dead assays, and one-way ANOVA with Tukey (GraphPad Prism). No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "repeated at least three times" sin ninguna justificacion del numero. Queda Unclear, no Yes.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro portion (MC3T3-E1 cell viability/adhesion on HG/XG/WG chitosan gels) is well described: aims clear, 'all experiments repeated at least three times', defined comparison groups and controls, standardized CCK-8/live-dead assays, and one-way ANOVA with Tukey (GraphPad Prism). No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "repeated at least three times" sin ninguna justificacion del numero. Queda Unclear, no Yes.]</t>
         </is>
       </c>
       <c r="Q54" t="n">
@@ -5299,7 +5300,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Osteoblasts were isolated from newborn SD rat cranial bones as a primary-cell source but were only used in vitro (adhesion rate, ALP/Alizarin Red staining on scaffold discs, n=3); no live-animal implantation or intervention was performed, so this is classified as in vitro. Aims, orthogonal-design comparison groups, standardized assays and Student's t-test statistics are clearly reported; no operator, randomization of group allocation, assessor, or blinding details given. [Correccion Q2 tras revision del texto completo, 2026-10-18: Declara n=3 "to decrease experimental errors", una razon generica sin calculo ni referencia real. Queda Unclear, no Yes.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Osteoblasts were isolated from newborn SD rat cranial bones as a primary-cell source but were only used in vitro (adhesion rate, ALP/Alizarin Red staining on scaffold discs, n=3); no live-animal implantation or intervention was performed, so this is classified as in vitro. Aims, orthogonal-design comparison groups, standardized assays and Student's t-test statistics are clearly reported; no operator, randomization of group allocation, assessor, or blinding details given. [Correccion Q2 tras revision del texto completo, 2026-10-18: Declara n=3 "to decrease experimental errors", una razon generica sin calculo ni referencia real. Queda Unclear, no Yes.]</t>
         </is>
       </c>
       <c r="Q55" t="n">
@@ -5389,7 +5390,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Melt-electrowritten PCL scaffold study with MC3T3-E1 cells: clear aims, explicit n=6 replicate samples, defined comparison groups (mPCL vs rPCL 1/3/5/7h, TCP/Triton controls), standardized LDH/CCK-8/Alizarin Red/ALP assays, and Student's t-test statistics with exact p-value thresholds. No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "6 different samples" sin justificacion del numero.] [Correccion Q11 tras revision del texto completo, 2026-10-18: No se identifica el nombre del software estadistico (solo "Student's t-test"); bajo el criterio estricto, queda Unclear, no Yes.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Melt-electrowritten PCL scaffold study with MC3T3-E1 cells: clear aims, explicit n=6 replicate samples, defined comparison groups (mPCL vs rPCL 1/3/5/7h, TCP/Triton controls), standardized LDH/CCK-8/Alizarin Red/ALP assays, and Student's t-test statistics with exact p-value thresholds. No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "6 different samples" sin justificacion del numero.] [Correccion Q11 tras revision del texto completo, 2026-10-18: No se identifica el nombre del software estadistico (solo "Student's t-test"); bajo el criterio estricto, queda Unclear, no Yes.]</t>
         </is>
       </c>
       <c r="Q56" t="n">
@@ -5479,7 +5480,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>Clear aims, detailed fabrication/assay methods, a defined control group (unmodified fiber/hydrogel composite), and appropriate statistics (ANOVA/Tukey, SPSS) are reported, but there is no sample-size justification, no description of randomization/allocation, no operator details, and no assessor blinding/inter-rater reliability for the cell studies. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Clear aims, detailed fabrication/assay methods, a defined control group (unmodified fiber/hydrogel composite), and appropriate statistics (ANOVA/Tukey, SPSS) are reported, but there is no sample-size justification, no description of randomization/allocation, no operator details, and no assessor blinding/inter-rater reliability for the cell studies.</t>
         </is>
       </c>
       <c r="Q57" t="n">
@@ -5569,7 +5570,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>Very thorough and well-controlled in vitro methodology (multiple neural cell types, MXene-free/inert and low/medium/high-density controls, validated assays, detailed GraphPad Prism statistics with reported n's), but randomization/allocation of samples to groups, operator identity, and blinding of outcome assessors (e.g., manual neurite-length measurement) are not described anywhere in the 20-page article. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Very thorough and well-controlled in vitro methodology (multiple neural cell types, MXene-free/inert and low/medium/high-density controls, validated assays, detailed GraphPad Prism statistics with reported n's), but randomization/allocation of samples to groups, operator identity, and blinding of outcome assessors (e.g., manual neurite-length measurement) are not described anywhere in the 20-page article.</t>
         </is>
       </c>
       <c r="Q58" t="n">
@@ -5659,7 +5660,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>Aims, fabrication protocol, and a formulation series with a comparator (conventional-mixing AL-CH-NC4H vs biopen-processed samples) are clearly described, with one-way ANOVA/Tukey statistics reported, but sample-size justification, randomization, operator, and blinding/assessor-reliability details are absent. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Aims, fabrication protocol, and a formulation series with a comparator (conventional-mixing AL-CH-NC4H vs biopen-processed samples) are clearly described, with one-way ANOVA/Tukey statistics reported, but sample-size justification, randomization, operator, and blinding/assessor-reliability details are absent.</t>
         </is>
       </c>
       <c r="Q59" t="n">
@@ -5749,7 +5750,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>Clear aims, a well-described PVA/OPP/HAp formulation series with an explicit control (1PVA/0OPP/HAp) and n=3 replicates, and standardized MTT/fluorescence assays are reported, but no statistical test is explicitly named despite significance asterisks appearing in some figures, and sample-size justification, randomization, and blinding/assessor details are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Clear aims, a well-described PVA/OPP/HAp formulation series with an explicit control (1PVA/0OPP/HAp) and n=3 replicates, and standardized MTT/fluorescence assays are reported, but no statistical test is explicitly named despite significance asterisks appearing in some figures, and sample-size justification, randomization, and blinding/assessor details are not reported.</t>
         </is>
       </c>
       <c r="Q60" t="n">
@@ -5929,7 +5930,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>Statistically sophisticated analysis (Shapiro-Wilk/Levene normality and variance testing, appropriately chosen parametric/non-parametric tests) and clear positive/negative controls (pure PCL, NC/PC) are reported, but no information on sample allocation/randomization, operator identity, or blinding of assessors is given. Note: MRI and immune-response/antibacterial testing were performed on scaffolds in vitro/in agar phantoms, not in a living animal, so this is classified as in vitro despite discussion of future in vivo/clinical use. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Statistically sophisticated analysis (Shapiro-Wilk/Levene normality and variance testing, appropriately chosen parametric/non-parametric tests) and clear positive/negative controls (pure PCL, NC/PC) are reported, but no information on sample allocation/randomization, operator identity, or blinding of assessors is given. Note: MRI and immune-response/antibacterial testing were performed on scaffolds in vitro/in agar phantoms, not in a living animal, so this is classified as in vitro despite discussion of future in vivo/clinical use.</t>
         </is>
       </c>
       <c r="Q62" t="n">
@@ -6019,7 +6020,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>Clear aims, detailed nanoneedle-array fabrication methods, TCP/PDA comparator groups, and defined statistics (SPSS, Student's t-test) are reported with n≥3-4, but sample-size justification, randomization, operator, and assessor-blinding details are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Clear aims, detailed nanoneedle-array fabrication methods, TCP/PDA comparator groups, and defined statistics (SPSS, Student's t-test) are reported with n≥3-4, but sample-size justification, randomization, operator, and assessor-blinding details are not reported.</t>
         </is>
       </c>
       <c r="Q63" t="n">
@@ -6109,7 +6110,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>Identity check: this file, labelled W34, was closely scrutinized given the known prior mislabeling issue for this study ID; title, authors, journal (Materials 2026, 19, 412) and abstract content (PVA/CS/HA/BA nanofibers, boric acid, antifungal activity for immunocompromised patients) match the expected citation exactly, so this is CONFIRMED as the correct paper. QUIN: clear aims, detailed electrospinning/crosslinking methods, a formulation series (PVA-CS, +HA, +0.25BA, +0.5BA) with ANOVA/Tukey statistics (GraphPad Prism) are reported, but sample-size justification (n=3 triplicate only), randomization, operator, and blinding/assessor details are absent. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Identity check: this file, labelled W34, was closely scrutinized given the known prior mislabeling issue for this study ID; title, authors, journal (Materials 2026, 19, 412) and abstract content (PVA/CS/HA/BA nanofibers, boric acid, antifungal activity for immunocompromised patients) match the expected citation exactly, so this is CONFIRMED as the correct paper. QUIN: clear aims, detailed electrospinning/crosslinking methods, a formulation series (PVA-CS, +HA, +0.25BA, +0.5BA) with ANOVA/Tukey statistics (GraphPad Prism) are reported, but sample-size justification (n=3 triplicate only), randomization, operator, and blinding/assessor details are absent.</t>
         </is>
       </c>
       <c r="Q64" t="n">
@@ -6199,7 +6200,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>Title/authors match the expected citation exactly; the journal name in the master table ('J Iron Sea Ind') appears to be a garbled/incorrect transcription — the actual journal is 'Collagen and Leather' (2024) 6:27, but this is clearly the same paper (identical title and author list), so CONFIRMED rather than MISMATCH. In vitro component: clear aims, detailed ink/printing methods, MG-63 cell attachment/morphology studies with ANOVA statistics reported, but no sample-size justification, randomization, operator, or blinding details. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Title/authors match the expected citation exactly; the journal name in the master table ('J Iron Sea Ind') appears to be a garbled/incorrect transcription — the actual journal is 'Collagen and Leather' (2024) 6:27, but this is clearly the same paper (identical title and author list), so CONFIRMED rather than MISMATCH. In vitro component: clear aims, detailed ink/printing methods, MG-63 cell attachment/morphology studies with ANOVA statistics reported, but no sample-size justification, randomization, operator, or blinding details.</t>
         </is>
       </c>
       <c r="Q65" t="n">
@@ -6379,7 +6380,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>Clear aims, very detailed nanoparticle/nanofiber synthesis and characterization methods, and consistent pure-PCL controls throughout are reported (CCK-8, live/dead, FACS, ICC), but no statistical test is explicitly named in the methods despite significance markers in figures, and sample-size justification, randomization, and blinding/assessor details are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Clear aims, very detailed nanoparticle/nanofiber synthesis and characterization methods, and consistent pure-PCL controls throughout are reported (CCK-8, live/dead, FACS, ICC), but no statistical test is explicitly named in the methods despite significance markers in figures, and sample-size justification, randomization, and blinding/assessor details are not reported.</t>
         </is>
       </c>
       <c r="Q67" t="n">
@@ -6469,7 +6470,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>Identity check: this file, labelled W43, was closely scrutinized given the known prior mislabeling issue for this study ID; title, authors, and journal (ACS Appl. Nano Mater. 2024, 7, 1245-1256) exactly match the expected citation (G vs GQD-reinforced PCL bone scaffolds), so this is CONFIRMED. QUIN: clear aims, detailed scaffold fabrication/characterization, a PCL-only control, and explicit one-way ANOVA with Tukey post hoc statistics are reported (n≥3), but sample-size justification, randomization, operator, and blinding/assessor-reliability details are absent. The authors themselves note this is a foundation for 'future in vivo studies', confirming no animal work was done here. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Identity check: this file, labelled W43, was closely scrutinized given the known prior mislabeling issue for this study ID; title, authors, and journal (ACS Appl. Nano Mater. 2024, 7, 1245-1256) exactly match the expected citation (G vs GQD-reinforced PCL bone scaffolds), so this is CONFIRMED. QUIN: clear aims, detailed scaffold fabrication/characterization, a PCL-only control, and explicit one-way ANOVA with Tukey post hoc statistics are reported (n≥3), but sample-size justification, randomization, operator, and blinding/assessor-reliability details are absent. The authors themselves note this is a foundation for 'future in vivo studies', confirming no animal work was done here.</t>
         </is>
       </c>
       <c r="Q68" t="n">
@@ -6739,7 +6740,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>In vitro osteoblast (MC3T3-E1) and antibacterial (P. gingivalis) assays use standardized commercial kits and ANOVA/Tukey statistics, but no sample-size justification, randomization, or blinding of operators/assessors is reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro osteoblast (MC3T3-E1) and antibacterial (P. gingivalis) assays use standardized commercial kits and ANOVA/Tukey statistics, but no sample-size justification, randomization, or blinding of operators/assessors is reported.</t>
         </is>
       </c>
       <c r="Q71" t="n">
@@ -6829,7 +6830,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>MG-63/HSF cell viability and osteogenic marker assays use standardized commercial kits (WST-1, ALP, OCN, TRAcP) and SPSS/ANOVA statistics; however sample-size justification, randomization/allocation of specimens, and operator/assessor blinding are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MG-63/HSF cell viability and osteogenic marker assays use standardized commercial kits (WST-1, ALP, OCN, TRAcP) and SPSS/ANOVA statistics; however sample-size justification, randomization/allocation of specimens, and operator/assessor blinding are not reported.</t>
         </is>
       </c>
       <c r="Q72" t="n">
@@ -6919,7 +6920,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>L929/BMSC cytotoxicity (CCK-8) and ALP osteogenic assays use commercial cell lines and a commercial hydroxyapatite (CHA) as control, with Prism/ANOVA statistics; however no sample-size justification, randomization, or blinding of operators/assessors is described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>L929/BMSC cytotoxicity (CCK-8) and ALP osteogenic assays use commercial cell lines and a commercial hydroxyapatite (CHA) as control, with Prism/ANOVA statistics; however no sample-size justification, randomization, or blinding of operators/assessors is described.</t>
         </is>
       </c>
       <c r="Q73" t="n">
@@ -7009,7 +7010,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>MG-63/BMSC assays (MTS, ALP, ARS) and mechanical testing (n=5 samples/group, tests replicated 3x) are clearly described with standardized methods and SPSS statistics, but no power/sample-size justification, randomization, or blinding is reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>MG-63/BMSC assays (MTS, ALP, ARS) and mechanical testing (n=5 samples/group, tests replicated 3x) are clearly described with standardized methods and SPSS statistics, but no power/sample-size justification, randomization, or blinding is reported.</t>
         </is>
       </c>
       <c r="Q74" t="n">
@@ -7099,7 +7100,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>BMSC cytocompatibility, antibacterial (E. coli/S. aureus), and qRT-PCR osteogenic gene expression assays are standardized with at least triplicate measurements and SPSS t-test/ANOVA statistics; however sample-size justification, randomization, and blinding are not reported. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>BMSC cytocompatibility, antibacterial (E. coli/S. aureus), and qRT-PCR osteogenic gene expression assays are standardized with at least triplicate measurements and SPSS t-test/ANOVA statistics; however sample-size justification, randomization, and blinding are not reported.</t>
         </is>
       </c>
       <c r="Q75" t="n">
@@ -7369,7 +7370,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>In vitro tenocyte culture (static and bioreactor dynamic culture) uses standardized assays (Live/Dead, qRT-PCR, IF) and SPSS ANOVA/LSD statistics with clear static-vs-dynamic comparison, but no sample-size justification, randomization, or blinding of operators/assessors is described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro tenocyte culture (static and bioreactor dynamic culture) uses standardized assays (Live/Dead, qRT-PCR, IF) and SPSS ANOVA/LSD statistics with clear static-vs-dynamic comparison, but no sample-size justification, randomization, or blinding of operators/assessors is described.</t>
         </is>
       </c>
       <c r="Q78" t="n">
@@ -7459,7 +7460,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>Fully in vitro PC-12 cell study (no live-animal SCI model despite the title's clinical framing). Clear aims, controls, detailed fabrication protocols, standardized instrumentation, and specified stats (GraphPad Prism, p&lt;0.05), but no sample-size justification, no operator details, no mention of randomization/blinding for cell seeding or image (ImageJ/flow cytometry) analysis, and PC-12 cell source/passage not stated. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Fully in vitro PC-12 cell study (no live-animal SCI model despite the title's clinical framing). Clear aims, controls, detailed fabrication protocols, standardized instrumentation, and specified stats (GraphPad Prism, p&lt;0.05), but no sample-size justification, no operator details, no mention of randomization/blinding for cell seeding or image (ImageJ/flow cytometry) analysis, and PC-12 cell source/passage not stated.</t>
         </is>
       </c>
       <c r="Q79" t="n">
@@ -7549,7 +7550,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>In vitro HUVEC work (survival, proliferation, VEGFR phosphorylation, morphology) is well described with clear controls and specified stats (one-way ANOVA/t-test, GraphPad Prism), and HUVEC source/passage range are given, but no sample-size justification (n=3 throughout, no power calc), no operator details, and no mention of randomization or blinding for any in vitro assay or image-based quantification. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>In vitro HUVEC work (survival, proliferation, VEGFR phosphorylation, morphology) is well described with clear controls and specified stats (one-way ANOVA/t-test, GraphPad Prism), and HUVEC source/passage range are given, but no sample-size justification (n=3 throughout, no power calc), no operator details, and no mention of randomization or blinding for any in vitro assay or image-based quantification.</t>
         </is>
       </c>
       <c r="Q80" t="n">
@@ -7639,7 +7640,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>Entirely in vitro (Saos-2 cell) study of a PHBV/PCL/diatom-frustule/melatonin scaffold; no in vivo work despite bone-regeneration framing. Clear aims, detailed fabrication/characterization methods, controls (TCPS, plain PHBV/PCL), and standardized assays (Alamar blue, ALP/BCA kits, SEM/EDX), with results in tables and graphs (mean±SD, significance letters). However, no explicit statistical-analysis subsection/test name was found despite significance markers being used, no sample-size justification (n=3), no operator details, and no mention of randomization or blinding for cell seeding or image-based (SEM/CLSM) analysis. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).]</t>
+          <t>Entirely in vitro (Saos-2 cell) study of a PHBV/PCL/diatom-frustule/melatonin scaffold; no in vivo work despite bone-regeneration framing. Clear aims, detailed fabrication/characterization methods, controls (TCPS, plain PHBV/PCL), and standardized assays (Alamar blue, ALP/BCA kits, SEM/EDX), with results in tables and graphs (mean±SD, significance letters). However, no explicit statistical-analysis subsection/test name was found despite significance markers being used, no sample-size justification (n=3), no operator details, and no mention of randomization or blinding for cell seeding or image-based (SEM/CLSM) analysis.</t>
         </is>
       </c>
       <c r="Q81" t="n">
@@ -7714,7 +7715,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAVEAT (added 2026-10-20, in response to external referee comment; CORRECTED 2026-10-20): D8 (incomplete outcome data), D9 (selective outcome reporting), and D10 (other sources of bias) were originally defaulted to 'Yes' when the primary text gave no explicit information, on the assumption that these domains presume freedom from bias absent contrary evidence. This default did NOT follow SYRCLE's own guidance, which specifies 'Unclear' when insufficient detail is reported to judge a domain -- silence should not be read as evidence of low risk. This has now been corrected by re-reading each study's Notes column (which records the primary-text evidence underlying every judgement) and recoding D8/D9/D10 to 'Unclear' wherever no concrete textual evidence supported 'Yes'; a 'Yes' is retained only where the Notes column documents specific supporting evidence (e.g., an explicit statement of complete outcome reporting, or an explicit funding/competing-interest declaration). The 'Overall risk judgement' column and the manuscript-level Low risk/Some concerns/High risk summary (Section 2.7) have been recomputed from these corrected values. Separately, an earlier annotation present in several Notes cells, tagged [CORREGIDO 2026-10-19], asserted that 'SYRCLE's standard convention is default=Yes (low risk) absent concrete evidence of a problem'; this claim has been verified against SYRCLE's primary source (Hooijmans et al., 2014) to be factually incorrect, and is superseded by this 2026-10-20 correction. See manuscript Section 2.7 and Discussion (Limitations) for full disclosure.</t>
+          <t>CAVEAT (added 2026-10-20): D8 (incomplete outcome data), D9 (selective outcome reporting), and D10 (other sources of bias) were originally defaulted to 'Yes' when the primary text gave no explicit information, on the assumption that these domains presume freedom from bias absent contrary evidence. This default did NOT follow SYRCLE's own guidance, which specifies 'Unclear' when insufficient detail is reported to judge a domain -- silence should not be read as evidence of low risk. This has now been corrected by re-reading each study's Notes column (which records the primary-text evidence underlying every judgement) and recoding D8/D9/D10 to 'Unclear' wherever no concrete textual evidence supported 'Yes'; a 'Yes' is retained only where the Notes column documents specific supporting evidence (e.g., an explicit statement of complete outcome reporting, or an explicit funding/competing-interest declaration). The 'Overall risk judgement' column and the manuscript-level Low risk/Some concerns/High risk summary (Section 2.7) have been recomputed from these corrected values. See manuscript Section 2.7 and Discussion (Limitations) for full disclosure.</t>
         </is>
       </c>
     </row>
@@ -7869,7 +7870,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Rabbit implantation study (n=3/timepoint, 12 rabbits total) states ARRIVE-guideline compliance and ethics approval and completely reports outcomes with no apparent attrition, but gives no information on randomization method, allocation concealment, animal housing, or blinding of caregivers/assessors (vessel counting used manual exclusion of false positives with no stated blinding). [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-20: D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rabbit implantation study (n=3/timepoint, 12 rabbits total) states ARRIVE-guideline compliance and ethics approval and completely reports outcomes with no apparent attrition, but gives no information on randomization method, allocation concealment, animal housing, or blinding of caregivers/assessors (vessel counting used manual exclusion of false positives with no stated blinding).</t>
         </is>
       </c>
     </row>
@@ -7941,7 +7942,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Rat random-skin-flap model with 5 groups (n=3 for histology) reports outcomes comprehensively with no apparent missing data, but no randomization method, allocation concealment, housing conditions, or blinding of caregivers/outcome assessors are described, and an ethics/IACUC approval statement was not found in the sections reviewed. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-20: D9 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rat random-skin-flap model with 5 groups (n=3 for histology) reports outcomes comprehensively with no apparent missing data, but no randomization method, allocation concealment, housing conditions, or blinding of caregivers/outcome assessors are described, and an ethics/IACUC approval statement was not found in the sections reviewed.</t>
         </is>
       </c>
     </row>
@@ -8013,7 +8014,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Mouse full-thickness wound study (40 mice, 4 groups, ethics-approved) reports all animals accounted for and outcomes fully described, but does not describe how mice were allocated to groups or to the day-7/day-14 subsets, nor housing conditions, allocation concealment, or blinding of caregivers/outcome assessors (H-SCORE, wound area measurement). [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-20: D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Mouse full-thickness wound study (40 mice, 4 groups, ethics-approved) reports all animals accounted for and outcomes fully described, but does not describe how mice were allocated to groups or to the day-7/day-14 subsets, nor housing conditions, allocation concealment, or blinding of caregivers/outcome assessors (H-SCORE, wound area measurement).</t>
         </is>
       </c>
     </row>
@@ -8085,7 +8086,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Rat full-thickness wound model uses a self-control design (treatment vs. control wound on the same animal, with baseline wound-size equivalence explicitly confirmed) and states animals were 'randomly euthanised' at each timepoint, which addresses baseline comparability and random timing of outcome assessment; however, allocation concealment, housing, caregiver/assessor blinding, and an ethics-approval statement were not found in the reviewed sections. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: diseno intra-animal confirmado en el texto primario (lado derecho=tratamiento, lado izquierdo=control del MISMO individuo). D2 (linea base) se marca Yes porque la equivalencia basal esta garantizada por diseno (mismo animal); D4 (alojamiento aleatorio) se marca Not applicable, no Yes/No, porque no existe una variable de alojamiento entre grupos que aleatorizar (ambos lados comparten el mismo animal y la misma jaula), igual que la convencion ya usada para el modelo CAM.] [CORREGIDO 2026-10-20: D8, D9 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rat full-thickness wound model uses a self-control design (treatment vs. control wound on the same animal, with baseline wound-size equivalence explicitly confirmed) and states animals were 'randomly euthanised' at each timepoint, which addresses baseline comparability and random timing of outcome assessment; however, allocation concealment, housing, caregiver/assessor blinding, and an ethics-approval statement were not found in the reviewed sections.</t>
         </is>
       </c>
     </row>
@@ -8157,7 +8158,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Rabbit bladder-defect implantation study (Sham, Control, BMHP, VP, BMHP+VP groups) is ethics-approved and reports outcomes fully with no apparent attrition, but does not describe the randomization method for group allocation, allocation concealment, housing, or blinding of caregivers/outcome assessors (immunofluorescence quantification of CD29/CD90/CD31). [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-20: D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rabbit bladder-defect implantation study (Sham, Control, BMHP, VP, BMHP+VP groups) is ethics-approved and reports outcomes fully with no apparent attrition, but does not describe the randomization method for group allocation, allocation concealment, housing, or blinding of caregivers/outcome assessors (immunofluorescence quantification of CD29/CD90/CD31).</t>
         </is>
       </c>
     </row>
@@ -8229,7 +8230,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Rat calvarial defect model with IACUC-equivalent ethics approval and randomly selected histology imaging fields, but no stated randomization method for group allocation, no allocation concealment, no blinding of caregivers or outcome assessors, and no reporting on attrition/exclusions. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rat calvarial defect model with IACUC-equivalent ethics approval and randomly selected histology imaging fields, but no stated randomization method for group allocation, no allocation concealment, no blinding of caregivers or outcome assessors, and no reporting on attrition/exclusions.</t>
         </is>
       </c>
     </row>
@@ -8301,7 +8302,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Rat (paired, within-animal, contralateral implantation) and miniature-pig wound models; no stated randomization of side/group allocation, no allocation concealment, no blinding of caregivers or assessors, and no attrition reporting, though animal protocols were institutionally approved. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-19: diseno intra-animal confirmado en el texto primario (lado derecho=tratamiento, lado izquierdo=control del MISMO individuo). D2 (linea base) se marca Yes porque la equivalencia basal esta garantizada por diseno (mismo animal); D4 (alojamiento aleatorio) se marca Not applicable, no Yes/No, porque no existe una variable de alojamiento entre grupos que aleatorizar (ambos lados comparten el mismo animal y la misma jaula), igual que la convencion ya usada para el modelo CAM.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rat (paired, within-animal, contralateral implantation) and miniature-pig wound models; no stated randomization of side/group allocation, no allocation concealment, no blinding of caregivers or assessors, and no attrition reporting, though animal protocols were institutionally approved.</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8374,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Rabbit tibial defect model: rats/rabbits were explicitly 'randomly allocated into four groups' and the study states ARRIVE-guideline compliance, but allocation concealment, random housing, blinding of caregivers/assessors and attrition reporting are not described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-19: D1 tenia 'Yes' por 'randomly allocated into four groups' sin metodo descrito (mismo bug ya corregido en P21/P28/P39/P47/W18; se habia omitido este estudio). Coincide ahora con la tabla del hermano. [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rabbit tibial defect model: rats/rabbits were explicitly 'randomly allocated into four groups' and the study states ARRIVE-guideline compliance, but allocation concealment, random housing, blinding of caregivers/assessors and attrition reporting are not described.</t>
         </is>
       </c>
     </row>
@@ -8445,7 +8446,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Rat cranial defect model: 48 rats were explicitly 'randomly divided into four groups' and the study states ARRIVE-guideline/IACUC compliance, but allocation concealment, random housing, blinding, random selection for outcome assessment and attrition are not described (n=6 per group per timepoint appears pre-set rather than randomly drawn from n=12). [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D1 estaba en 'Yes' porque el texto dice 'randomly divided/assigned/allocated' sin describir el metodo (sin numero aleatorio, tabla, sorteo ni software); bajo el criterio estricto ya aplicado a QUIN Q7 para este mismo estudio, esto es 'No'. Corregido para ser consistente.] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rat cranial defect model: 48 rats were explicitly 'randomly divided into four groups' and the study states ARRIVE-guideline/IACUC compliance, but allocation concealment, random housing, blinding, random selection for outcome assessment and attrition are not described (n=6 per group per timepoint appears pre-set rather than randomly drawn from n=12).</t>
         </is>
       </c>
     </row>
@@ -8517,7 +8518,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Rat traumatic brain injury/craniotomy model with IACUC approval, but no statement of randomization method, allocation concealment, blinding (including for Bederson motor-score assessment), or attrition handling. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rat traumatic brain injury/craniotomy model with IACUC approval, but no statement of randomization method, allocation concealment, blinding (including for Bederson motor-score assessment), or attrition handling.</t>
         </is>
       </c>
     </row>
@@ -8589,7 +8590,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Wistar rat calvaria defect model: rats were 'divided into three groups' (randomization method not explicitly named); study states ARRIVE-guideline compliance and includes a dedicated systemic-toxicity histopathology evaluation of major organs, but allocation concealment, blinding and attrition are still not described. Overall judgement harmonized to High risk on QC re-review (2026-09-24) for consistency with other studies presenting an identical all-Unclear domain profile (P15, P17, P22): ARRIVE-guideline compliance and the additional toxicology evaluation are not captured by the ten SYRCLE domains themselves, so an all-Unclear profile is rated High risk regardless of these external indicators. Originally rated Some concerns; changed by both risk-of-bias assessors after external audit flagged the inconsistency. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-19: diseno intra-animal confirmado en el texto primario (lado derecho=tratamiento, lado izquierdo=control del MISMO individuo). D2 (linea base) se marca Yes porque la equivalencia basal esta garantizada por diseno (mismo animal); D4 (alojamiento aleatorio) se marca Not applicable, no Yes/No, porque no existe una variable de alojamiento entre grupos que aleatorizar (ambos lados comparten el mismo animal y la misma jaula), igual que la convencion ya usada para el modelo CAM.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Wistar rat calvaria defect model: rats were 'divided into three groups' (randomization method not explicitly named); study states ARRIVE-guideline compliance and includes a dedicated systemic-toxicity histopathology evaluation of major organs, but allocation concealment, blinding and attrition are still not described. Overall judgement harmonized to High risk on QC re-review (2026-09-24) for consistency with other studies presenting an identical all-Unclear domain profile (P15, P17, P22): ARRIVE-guideline compliance and the additional toxicology evaluation are not captured by the ten SYRCLE domains themselves, so an all-Unclear profile is rated High risk regardless of these external indicators. Originally rated Some concerns; changed by both risk-of-bias assessors after external audit flagged the inconsistency.</t>
         </is>
       </c>
     </row>
@@ -8661,7 +8662,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Rat subcutaneous implantation model: 18 rats were explicitly 'randomly divided into three groups' and rats were explicitly 'randomly selected for euthanasia' at each timepoint, but allocation concealment, random housing, blinding of caregivers/assessors and attrition reporting are not described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D1 estaba en 'Yes' porque el texto dice 'randomly divided/assigned/allocated' sin describir el metodo (sin numero aleatorio, tabla, sorteo ni software); bajo el criterio estricto ya aplicado a QUIN Q7 para este mismo estudio, esto es 'No'. Corregido para ser consistente.] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rat subcutaneous implantation model: 18 rats were explicitly 'randomly divided into three groups' and rats were explicitly 'randomly selected for euthanasia' at each timepoint, but allocation concealment, random housing, blinding of caregivers/assessors and attrition reporting are not described.</t>
         </is>
       </c>
     </row>
@@ -8733,7 +8734,7 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Subcutaneous (n=6) and in situ cartilage-defect (n=40) SD rat experiments report ethical approval and group sizes, but do not describe allocation sequence generation, allocation concealment, random housing, blinding of caregivers/assessors, or how attrition/selective reporting were handled. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Subcutaneous (n=6) and in situ cartilage-defect (n=40) SD rat experiments report ethical approval and group sizes, but do not describe allocation sequence generation, allocation concealment, random housing, blinding of caregivers/assessors, or how attrition/selective reporting were handled.</t>
         </is>
       </c>
     </row>
@@ -8805,7 +8806,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>In vivo component is a small proof-of-concept demonstration (implants in a single mouse; two menisci implanted ex vivo in swine legs), with no randomization, allocation concealment, blinding, or group-level statistics reported for the animal work. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-20: D8, D9 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>In vivo component is a small proof-of-concept demonstration (implants in a single mouse; two menisci implanted ex vivo in swine legs), with no randomization, allocation concealment, blinding, or group-level statistics reported for the animal work.</t>
         </is>
       </c>
     </row>
@@ -8877,7 +8878,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>24 rats were explicitly randomly assigned to 4 groups (calvarial defect model) with ethics approval, but allocation concealment, random housing, blinding of surgeons/caregivers, blinded outcome assessment, and attrition handling are not described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D1 estaba en 'Yes' porque el texto dice 'randomly divided/assigned/allocated' sin describir el metodo (sin numero aleatorio, tabla, sorteo ni software); bajo el criterio estricto ya aplicado a QUIN Q7 para este mismo estudio, esto es 'No'. Corregido para ser consistente.] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>24 rats were explicitly randomly assigned to 4 groups (calvarial defect model) with ethics approval, but allocation concealment, random housing, blinding of surgeons/caregivers, blinded outcome assessment, and attrition handling are not described.</t>
         </is>
       </c>
     </row>
@@ -8949,7 +8950,7 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>24 SD rats were randomly allocated to 4 groups for a cranial critical-size defect model, and three rats per group were randomly selected for euthanasia at each timepoint, but allocation concealment, random housing, and blinding of caregivers/outcome assessors (Micro-CT, histology) are not described, and attrition/selective-reporting handling is not addressed. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D1 estaba en 'Yes' porque el texto dice 'randomly divided/assigned/allocated' sin describir el metodo (sin numero aleatorio, tabla, sorteo ni software); bajo el criterio estricto ya aplicado a QUIN Q7 para este mismo estudio, esto es 'No'. Corregido para ser consistente.] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>24 SD rats were randomly allocated to 4 groups for a cranial critical-size defect model, and three rats per group were randomly selected for euthanasia at each timepoint, but allocation concealment, random housing, and blinding of caregivers/outcome assessors (Micro-CT, histology) are not described, and attrition/selective-reporting handling is not addressed.</t>
         </is>
       </c>
     </row>
@@ -9021,7 +9022,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>IACUC-approved diabetic-rat wound model with n=10/group stated as 'randomly divided', but the randomization method, allocation concealment, blinding of caregivers/assessors, and random housing/selection are not described anywhere in the methods. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>IACUC-approved diabetic-rat wound model with n=10/group stated as 'randomly divided', but the randomization method, allocation concealment, blinding of caregivers/assessors, and random housing/selection are not described anywhere in the methods.</t>
         </is>
       </c>
     </row>
@@ -9093,7 +9094,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Rats were explicitly randomly assigned to 4 equal groups (n=10) in a distal femur defect model with adequate sample size and complete outcome reporting, but allocation concealment, randomized housing, and blinding of caregivers/outcome assessors were not described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: PDF de Huang et al. 2024 (IJN) ya conseguido y verificado. El texto dice 'Forty...SD rats were randomly assigned to four groups of equal numbers' sin describir el metodo de aleatorizacion (sin numero aleatorio, tabla, sorteo ni software). Bajo el criterio estricto ya establecido, D1=No, no Yes. Coincide ahora con la tabla del hermano.] [CORREGIDO 2026-10-20: D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rats were explicitly randomly assigned to 4 equal groups (n=10) in a distal femur defect model with adequate sample size and complete outcome reporting, but allocation concealment, randomized housing, and blinding of caregivers/outcome assessors were not described.</t>
         </is>
       </c>
     </row>
@@ -9165,7 +9166,7 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Mouse air-pouch model (n=20 Balb/C mice, IACUC-approved) implanted with E0/E3 scaffolds and given peritoneal fluorescent-magnetic particles. No description of allocation sequence generation, allocation concealment, random housing, caregiver/assessor blinding, random selection for outcome assessment, or explicit handling of attrition. Outcome reporting appears complete (histology, PCR, fluorescence) and funder is stated to have had no role in study design/analysis/writing. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D9 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Mouse air-pouch model (n=20 Balb/C mice, IACUC-approved) implanted with E0/E3 scaffolds and given peritoneal fluorescent-magnetic particles. No description of allocation sequence generation, allocation concealment, random housing, caregiver/assessor blinding, random selection for outcome assessment, or explicit handling of attrition. Outcome reporting appears complete (histology, PCR, fluorescence) and funder is stated to have had no role in study design/analysis/writing.</t>
         </is>
       </c>
     </row>
@@ -9237,7 +9238,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>36 SD rats subcutaneously implanted with gel scaffolds, explicitly 'randomly divided into 3 groups' (method not specified) with random selection of 4 rats/group for euthanasia at each of 2/4/8-week timepoints. No description of allocation concealment, random housing, or blinding of caregivers/assessors; baseline similarity and freedom from attrition not explicitly confirmed. Outcome reporting (H&amp;E, Masson trichrome) appears complete; conflict-of-interest/funding statement not seen in pages reviewed. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D1 estaba en 'Yes' porque el texto dice 'randomly divided/assigned/allocated' sin describir el metodo (sin numero aleatorio, tabla, sorteo ni software); bajo el criterio estricto ya aplicado a QUIN Q7 para este mismo estudio, esto es 'No'. Corregido para ser consistente.] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-19: D10 decia 'conflicto de interes/financiamiento no visto en paginas revisadas', pero el texto SI tiene 'Declaration of competing interest: ...no known competing financial [interests]' y una seccion de Funding explicita (pag. revisada mas completa). Corregido a Yes. [CORREGIDO 2026-10-20: D8, D9 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>36 SD rats subcutaneously implanted with gel scaffolds, explicitly 'randomly divided into 3 groups' (method not specified) with random selection of 4 rats/group for euthanasia at each of 2/4/8-week timepoints. No description of allocation concealment, random housing, or blinding of caregivers/assessors; baseline similarity and freedom from attrition not explicitly confirmed. Outcome reporting (H&amp;E, Masson trichrome) appears complete; conflict-of-interest/funding statement not seen in pages reviewed.</t>
         </is>
       </c>
     </row>
@@ -9309,7 +9310,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Modelo murino de herida infectada con S. aureus (BALB/c hembra, 4 grupos: PBS, NIR, NPs, NPs+NIR). El texto dice '6 mice... fueron divididos en cuatro grupos', numero de animales por grupo ambiguo/muy bajo. Sin metodo de aleatorizacion, ocultamiento de asignacion, cegamiento de cuidadores o evaluadores, ni manejo de datos incompletos descritos explicitamente; el reporte de resultados parece completo (area de herida, histologia, CD31/VEGF) sin senales de reporte selectivo. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Modelo murino de herida infectada con S. aureus (BALB/c hembra, 4 grupos: PBS, NIR, NPs, NPs+NIR). El texto dice '6 mice... fueron divididos en cuatro grupos', numero de animales por grupo ambiguo/muy bajo. Sin metodo de aleatorizacion, ocultamiento de asignacion, cegamiento de cuidadores o evaluadores, ni manejo de datos incompletos descritos explicitamente; el reporte de resultados parece completo (area de herida, histologia, CD31/VEGF) sin senales de reporte selectivo.</t>
         </is>
       </c>
     </row>
@@ -9381,7 +9382,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>9 New Zealand white rabbits were explicitly 'randomly divided into three groups' (D1: Yes), but allocation concealment, randomized housing, blinding of caregivers/surgeons and outcome assessors (micro-CT/histology), random selection for outcome assessment, and handling of attrition are not reported. With only 3 rabbits per scaffold group evaluated across 3 time points (4/8/12 weeks), per-timepoint group sizes appear very small and attrition/exclusions are not explicitly addressed. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>9 New Zealand white rabbits were explicitly 'randomly divided into three groups' (D1: Yes), but allocation concealment, randomized housing, blinding of caregivers/surgeons and outcome assessors (micro-CT/histology), random selection for outcome assessment, and handling of attrition are not reported. With only 3 rabbits per scaffold group evaluated across 3 time points (4/8/12 weeks), per-timepoint group sizes appear very small and attrition/exclusions are not explicitly addressed.</t>
         </is>
       </c>
     </row>
@@ -9453,7 +9454,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Rat calvarial defect study (24 male Sprague-Dawley rats, 4 groups, IACUC-approved) reports complete outcome data (micro-CT, histology, IHC at 4 and 8 weeks) with no evidence of selective reporting, but does not describe the randomization method, allocation concealment, random housing, or blinding of caregivers/outcome assessors, so most domains cannot be judged. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rat calvarial defect study (24 male Sprague-Dawley rats, 4 groups, IACUC-approved) reports complete outcome data (micro-CT, histology, IHC at 4 and 8 weeks) with no evidence of selective reporting, but does not describe the randomization method, allocation concealment, random housing, or blinding of caregivers/outcome assessors, so most domains cannot be judged.</t>
         </is>
       </c>
     </row>
@@ -9525,7 +9526,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Sprague Dawley rats with femoral bone defects were 'randomly grafted' with materials (6 samples/group), but no randomization method, allocation concealment, blinding, random housing, or explicit attrition/completion statement is reported for the in vivo arm. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Sprague Dawley rats with femoral bone defects were 'randomly grafted' with materials (6 samples/group), but no randomization method, allocation concealment, blinding, random housing, or explicit attrition/completion statement is reported for the in vivo arm.</t>
         </is>
       </c>
     </row>
@@ -9597,7 +9598,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>In-ovo CAM angiogenesis assay (fertilized chick eggs, triplicate per group, ethically approved) reports complete vessel-density and histological outcomes with no evidence of selective reporting, but egg allocation/randomization method, blinding of vessel-counting assessors, and embryo attrition are not described. Domains D4 (random housing) and D5 (caregiver blinding) are not clearly applicable to a CAM model and are marked Unclear on that basis. [D4 marked N/A, not Unclear/No: a CAM (egg) model has no animal-housing concept; domain excluded from this study's overall-judgement profile.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>In-ovo CAM angiogenesis assay (fertilized chick eggs, triplicate per group, ethically approved) reports complete vessel-density and histological outcomes with no evidence of selective reporting, but egg allocation/randomization method, blinding of vessel-counting assessors, and embryo attrition are not described. Domains D4 (random housing) and D5 (caregiver blinding) are not clearly applicable to a CAM model and are marked Unclear on that basis. [D4 marked N/A, not Unclear/No: a CAM (egg) model has no animal-housing concept; domain excluded from this study's overall-judgement profile.]</t>
         </is>
       </c>
     </row>
@@ -9669,7 +9670,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Rabbit Achilles tendon defect model (cellular vs. acellular scaffold) and nude mouse subcutaneous implantation are used, but group allocation method, allocation concealment, random housing, blinding of caregivers and of the histological/adhesion scorer, and explicit attrition reporting are not described. [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D9, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Rabbit Achilles tendon defect model (cellular vs. acellular scaffold) and nude mouse subcutaneous implantation are used, but group allocation method, allocation concealment, random housing, blinding of caregivers and of the histological/adhesion scorer, and explicit attrition reporting are not described.</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9742,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Chick chorioallantoic membrane (CAM) assay, n=10 eggs/condition; a partial in-ovo model rather than a full live-animal study. No allocation/randomization method, allocation concealment, or blinding (caregiver or assessor) is reported for scaffold placement or ImageJ-based vessel quantification; several domains (random housing, random selection for assessment) are not clearly applicable to a CAM model. Reported outcomes (vessel area, vessel number) appear completely reported (D9=Yes); no attrition/exclusions mentioned but not explicitly addressed either way. Authors' ethics statement confirms only CAM assay was performed, no live-animal experiments. [D4 marked N/A, not Unclear/No: a CAM (egg) model has no animal-housing concept; domain excluded from this study's overall-judgement profile.] [Armonizacion 2026-10-18: Unclear recodificado como No; escala Yes/No unica en ambas tablas (propia y de hermano).] [CORREGIDO 2026-10-19: D8/D9/D10 preguntan si el estudio esta LIBRE de ese sesgo (no si se describio una salvaguarda); la convencion SYRCLE estandar es default=Yes (bajo riesgo) salvo evidencia concreta de un problema. La conversion Unclear-&gt;No aplicada el 2026-10-18 fue incorrecta para estos 3 dominios; se corrige aqui a Unclear/No-sin-evidencia -&gt; Yes, manteniendo No solo donde hay evidencia especifica de un problema real.] [CORREGIDO 2026-10-20: D8, D10 recodificado(s) de 'Yes' a 'Unclear' -- el 'Yes' por defecto no seguia la guia propia de SYRCLE y no estaba evidenciado en el texto primario citado en esta nota; ver tambien la nota [CORREGIDO 2026-10-19] en esta misma celda, cuya premisa (default SYRCLE = Yes) se ha verificado que es incorrecta.]</t>
+          <t>Chick chorioallantoic membrane (CAM) assay, n=10 eggs/condition; a partial in-ovo model rather than a full live-animal study. No allocation/randomization method, allocation concealment, or blinding (caregiver or assessor) is reported for scaffold placement or ImageJ-based vessel quantification; several domains (random housing, random selection for assessment) are not clearly applicable to a CAM model. Reported outcomes (vessel area, vessel number) appear completely reported (D9=Yes); no attrition/exclusions mentioned but not explicitly addressed either way. Authors' ethics statement confirms only CAM assay was performed, no live-animal experiments. [D4 marked N/A, not Unclear/No: a CAM (egg) model has no animal-housing concept; domain excluded from this study's overall-judgement profile.]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix S3 outcome-summary truncation and remove internal Spanish/provenance notes from S5
</commit_message>
<xml_diff>
--- a/supplementary/Supplementary_Table_S5_Risk_of_Bias_QUIN_SYRCLE.xlsx
+++ b/supplementary/Supplementary_Table_S5_Risk_of_Bias_QUIN_SYRCLE.xlsx
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Delemeester et al., 2024, Adv Funct Mater [recuperado en 2da subida]</t>
+          <t>Delemeester et al., 2024, Adv Funct Mater</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ucan et al., 2025, Macromol Mater Eng [recuperado en 2da subida]</t>
+          <t>Ucan et al., 2025, Macromol Mater Eng</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Liu et al., 2025, Small Structures [recuperado en 2da subida]</t>
+          <t>Liu et al., 2025, Small Structures</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Unusually rigorous statistical framework (mixed-effects models, plate-level random effects, Cohen's d, one-sample t-tests vs ISO threshold, minimum 4 replicates justified by regulatory design), but operator identity/training, randomization of sample allocation, and blinding of outcome assessment are not reported. [Correccion Q11 tras revision del texto completo, 2026-10-18: No se identifica el nombre del software estadistico (solo ANOVA, Tukey HSD, Cohen's d, modelo mixto); bajo el criterio estricto acordado (Q11 requiere software nombrado), queda Unclear, no Yes.]</t>
+          <t>Unusually rigorous statistical framework (mixed-effects models, plate-level random effects, Cohen's d, one-sample t-tests vs ISO threshold, minimum 4 replicates justified by regulatory design), but operator identity/training, randomization of sample allocation, and blinding of outcome assessment are not reported. For Q11, no statistical software name is identified (only the test names — ANOVA, Tukey HSD, Cohen's d, mixed model — are given); under the criterion applied here (Q11 requires the software itself to be named), this remains Unclear rather than Yes.</t>
         </is>
       </c>
       <c r="Q37" t="n">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Huang et al., 2024, Int J Nanomedicine [recuperado en 2da subida]</t>
+          <t>Huang et al., 2024, Int J Nanomedicine</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -4419,7 +4419,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Zhu et al., 2024, International Journal of Biological Macromolecules [recuperado en 2da subida]</t>
+          <t>Zhu et al., 2024, International Journal of Biological Macromolecules</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>Clear aims, methods, controls (2D mat/dropcast/PTP), stated replicate number (n=6) and ANOVA/Tukey statistics with exact p-values. No mention of operator details, randomization of well allocation, assessor blinding, or inter-rater reliability, which are the main gaps. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "n = 6" sin ninguna justificacion numerica o estadistica de por que se elige ese tamano; no hay calculo de poder ni referencia a un estandar. Bajo el criterio estricto (Q2 requiere justificacion real, no solo declarar el numero de replicas), queda Unclear, no Yes.]</t>
+          <t>Clear aims, methods, controls (2D mat/dropcast/PTP), stated replicate number (n=6) and ANOVA/Tukey statistics with exact p-values. No mention of operator details, randomization of well allocation, assessor blinding, or inter-rater reliability, which are the main gaps. For Q2, only "n = 6" is stated, with no numerical or statistical justification for that choice, no power calculation, and no reference to a standard; under the criterion applied here (Q2 requires a genuine justification, not merely stating the replicate count), this remains Unclear rather than Yes.</t>
         </is>
       </c>
       <c r="Q47" t="n">
@@ -4599,7 +4599,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Peng et al., 2024, Materials Letters 361:135922 (HA whisker w/ Mg/Sr ions) [ID RECOVERED FROM MISLABELED FILE - see note]</t>
+          <t>Peng et al., 2024, Materials Letters 361:135922 (HA whisker w/ Mg/Sr ions)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -4669,7 +4669,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>The file under W03 is a different, much shorter paper (Materials Letters short communication) on Mg/Sr-modified hydroxyapatite whisker scaffolds, not the expected Zhu et al. cellulose-nanocrystal/HA/PVA paper. Methods are minimal: no cell source/passage details, no stated replicate numbers for CCK-8/ALP, no statistical test named anywhere, and ALP results shown only as unquantified images. | RECOVERY NOTE: This is the TRUE W07 study content, found inside a file that was incorrectly named "W03.pdf". The W03.pdf filename does not contain the real W03 study (Zhu et al., cellulose nanocrystal/HA/PVA), which is still missing.</t>
+          <t>The PDF file originally labeled as Study W03 was found to contain a different, shorter paper (a Materials Letters short communication on Mg/Sr-modified hydroxyapatite whisker scaffolds) rather than the intended Zhu et al. cellulose-nanocrystal/HA/PVA study. That content is assessed here under Study ID W07, matching its actual citation; the Zhu et al. study originally intended for W03 remains to be located. Methods in this file are minimal: no cell source/passage details, no stated replicate numbers for CCK-8/ALP, no statistical test named, and ALP results are shown only as unquantified images.</t>
         </is>
       </c>
       <c r="Q48" t="n">
@@ -4689,7 +4689,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Najar et al., 2024, Materials Today Materialia [recuperado en 2da subida]</t>
+          <t>Najar et al., 2024, Materials Today Materialia</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>In vitro portion (BMSC osteoblast induction, SBF degradation, alamarBlue proliferation) has clear aims, groups (E0-E4), triplicate-combined statistics (t-test/ANOVA), and adequately presented results. No operator, randomization, assessor, or blinding details given. [Correccion Q2 tras revision del texto completo, 2026-10-18: El calculo de tamano de muestra con el programa PSTM se aplica explicitamente "the sample size of the animal experiment" (SYRCLE/in vivo), no a la porcion in vitro, que solo declara "3 individual experiments... combined for statistical analysis" sin justificacion propia. Para QUIN (in vitro) queda Unclear, no Yes.]</t>
+          <t>In vitro portion (BMSC osteoblast induction, SBF degradation, alamarBlue proliferation) has clear aims, groups (E0-E4), triplicate-combined statistics (t-test/ANOVA), and adequately presented results. No operator, randomization, assessor, or blinding details given. For Q2, the PSTM-based sample-size calculation reported in the source text is stated explicitly for "the sample size of the animal experiment" (the SYRCLE/in vivo portion), not for the in vitro portion, which only states "3 individual experiments... combined for statistical analysis" without its own justification. For QUIN (in vitro), this remains Unclear rather than Yes.</t>
         </is>
       </c>
       <c r="Q50" t="n">
@@ -4959,7 +4959,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Wang et al., 2024, Colloids and Surfaces B: Biointerfaces [recuperado en 2da subida]</t>
+          <t>Wang et al., 2024, Colloids and Surfaces B: Biointerfaces</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>Well-reported core-shell electrospun scaffold study: clear aims, triplicate analyses stated ('all experimental analyses were conducted in triplicate'), defined comparison groups (0E/1E/3E/5E), standardized assays (MTT, qRT-PCR with defined primers) and two-way ANOVA with GraphPad Prism. No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Declara "triplicate to ensure statistical robustness" y n=3 segun ASTM D882 para el ensayo mecanico, pero no hay justificacion estadistica real (calculo de poder o referencia) de por que ese numero es adecuado; el estandar ASTM especifica el procedimiento, no justifica el tamano de muestra biologico. Queda Unclear, no Yes.]</t>
+          <t>Well-reported core-shell electrospun scaffold study: clear aims, triplicate analyses stated ('all experimental analyses were conducted in triplicate'), defined comparison groups (0E/1E/3E/5E), standardized assays (MTT, qRT-PCR with defined primers) and two-way ANOVA with GraphPad Prism. No operator, randomization, assessor, or blinding details reported. For Q2, the study states "triplicate to ensure statistical robustness" and n=3 per ASTM D882 for the mechanical test, but there is no genuine statistical justification (power calculation or reference) for why that number is adequate; the ASTM standard specifies the test procedure, not the biological sample size. This remains Unclear rather than Yes.</t>
         </is>
       </c>
       <c r="Q53" t="n">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>In vitro portion (MC3T3-E1 cell viability/adhesion on HG/XG/WG chitosan gels) is well described: aims clear, 'all experiments repeated at least three times', defined comparison groups and controls, standardized CCK-8/live-dead assays, and one-way ANOVA with Tukey (GraphPad Prism). No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "repeated at least three times" sin ninguna justificacion del numero. Queda Unclear, no Yes.]</t>
+          <t>In vitro portion (MC3T3-E1 cell viability/adhesion on HG/XG/WG chitosan gels) is well described: aims clear, 'all experiments repeated at least three times', defined comparison groups and controls, standardized CCK-8/live-dead assays, and one-way ANOVA with Tukey (GraphPad Prism). No operator, randomization, assessor, or blinding details reported. For Q2, only "repeated at least three times" is stated, with no justification for that number. This remains Unclear rather than Yes.</t>
         </is>
       </c>
       <c r="Q54" t="n">
@@ -5299,7 +5299,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>Osteoblasts were isolated from newborn SD rat cranial bones as a primary-cell source but were only used in vitro (adhesion rate, ALP/Alizarin Red staining on scaffold discs, n=3); no live-animal implantation or intervention was performed, so this is classified as in vitro. Aims, orthogonal-design comparison groups, standardized assays and Student's t-test statistics are clearly reported; no operator, randomization of group allocation, assessor, or blinding details given. [Correccion Q2 tras revision del texto completo, 2026-10-18: Declara n=3 "to decrease experimental errors", una razon generica sin calculo ni referencia real. Queda Unclear, no Yes.]</t>
+          <t>Osteoblasts were isolated from newborn SD rat cranial bones as a primary-cell source but were only used in vitro (adhesion rate, ALP/Alizarin Red staining on scaffold discs, n=3); no live-animal implantation or intervention was performed, so this is classified as in vitro. Aims, orthogonal-design comparison groups, standardized assays and Student's t-test statistics are clearly reported; no operator, randomization of group allocation, assessor, or blinding details given. For Q2, n=3 is justified only as "to decrease experimental errors" — a generic rationale with no calculation or real reference. This remains Unclear rather than Yes.</t>
         </is>
       </c>
       <c r="Q55" t="n">
@@ -5389,7 +5389,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>Melt-electrowritten PCL scaffold study with MC3T3-E1 cells: clear aims, explicit n=6 replicate samples, defined comparison groups (mPCL vs rPCL 1/3/5/7h, TCP/Triton controls), standardized LDH/CCK-8/Alizarin Red/ALP assays, and Student's t-test statistics with exact p-value thresholds. No operator, randomization, assessor, or blinding details reported. [Correccion Q2 tras revision del texto completo, 2026-10-18: Solo declara "6 different samples" sin justificacion del numero.] [Correccion Q11 tras revision del texto completo, 2026-10-18: No se identifica el nombre del software estadistico (solo "Student's t-test"); bajo el criterio estricto, queda Unclear, no Yes.]</t>
+          <t>Melt-electrowritten PCL scaffold study with MC3T3-E1 cells: clear aims, explicit n=6 replicate samples, defined comparison groups (mPCL vs rPCL 1/3/5/7h, TCP/Triton controls), standardized LDH/CCK-8/Alizarin Red/ALP assays, and Student's t-test statistics with exact p-value thresholds. No operator, randomization, assessor, or blinding details reported. For Q2, only "6 different samples" is stated, with no justification for that number. For Q11, no statistical software name is identified (only "Student's t-test" is named); under the criterion applied here, both remain Unclear rather than Yes.</t>
         </is>
       </c>
       <c r="Q56" t="n">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Zhang et al., 2023, Int J Biol Macromol [nota: titulo/revista de la tabla maestra difieren ligeramente - ver notas]</t>
+          <t>Zhang et al., 2023, Int J Biol Macromol (title/journal in Table S1 differs slightly for the same article; see Notes)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -5839,7 +5839,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>Titulo real: 'Multifunctional chitosan/alginate hydrogel incorporated with bioactive glass nanocomposites enabling photothermal and nitric oxide release activities for bacteria-infected wound healing' (Int J Biol Macromol 232:123445, 2023) - coincide en autor principal (Zhang) y en el sistema quitosano/alginato + polidopamina (PDA recubre las nanoparticulas de vidrio bioactivo), pero el titulo/revista de la Tabla S1 ('Polydopamine nanospheres modified chitosan/alginate hydrogel nanocomposites', J Macromol Sci) parece ser una paraphrasis/nombre de revista incorrecto del mismo articulo, no un estudio distinto. Metodologia, controles y estadistica (t-test, triplicado) bien reportados; faltan justificacion de tamano de muestra, detalles de operador, aleatorizacion y cegamiento.</t>
+          <t>Full title and journal: 'Multifunctional chitosan/alginate hydrogel incorporated with bioactive glass nanocomposites enabling photothermal and nitric oxide release activities for bacteria-infected wound healing' (Int J Biol Macromol 232:123445, 2023). This matches the lead author (Zhang) and the chitosan/alginate + polydopamine-coated bioactive-glass-nanoparticle system; the title/journal given in Supplementary Table S1 ('Polydopamine nanospheres modified chitosan/alginate hydrogel nanocomposites', J Macromol Sci) appears to be a paraphrased title and an incorrect journal name for the same article, not a different study. Methodology, controls, and statistics (t-test, triplicate) are well reported; sample-size justification, operator details, randomization, and blinding are not described.</t>
         </is>
       </c>
       <c r="Q61" t="n">
@@ -6219,7 +6219,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Weng et al., 2026, Dental Materials Journal [recuperado en 2da subida]</t>
+          <t>Weng et al., 2026, Dental Materials Journal</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -6489,7 +6489,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Pilli et al., 2025, Journal of Materials Research [recuperado en 2da subida]</t>
+          <t>Pilli et al., 2025, Journal of Materials Research</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -6579,7 +6579,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Zhao et al., 2022, Journal of Magnesium and Alloys [recuperado en 2da subida]</t>
+          <t>Zhao et al., 2022, Journal of Magnesium and Alloys</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -7119,7 +7119,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Pudełko-Prażuch et al., 2024, Journal of Functional Biomaterials [recuperado en 2da subida]</t>
+          <t>Pudełko-Prażuch et al., 2024, Journal of Functional Biomaterials</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Alizadeh &amp; Mahmoodi, 2025, Progress in Biomaterials [recuperado en 2da subida]</t>
+          <t>Alizadeh &amp; Mahmoodi, 2025, Progress in Biomaterials</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -8746,7 +8746,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Delemeester et al., 2024, Adv Funct Mater [recuperado en 2da subida]</t>
+          <t>Delemeester et al., 2024, Adv Funct Mater</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Huang et al., 2024, Int J Nanomedicine [recuperado en 2da subida]</t>
+          <t>Huang et al., 2024, Int J Nanomedicine</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -9250,7 +9250,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Zhang et al., 2023, Int J Biol Macromol [nota: titulo/revista de la tabla maestra difieren ligeramente - ver notas]</t>
+          <t>Zhang et al., 2023, Int J Biol Macromol (title/journal in Table S1 differs slightly for the same article; see Notes)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -9310,7 +9310,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Modelo murino de herida infectada con S. aureus (BALB/c hembra, 4 grupos: PBS, NIR, NPs, NPs+NIR). El texto dice '6 mice... fueron divididos en cuatro grupos', numero de animales por grupo ambiguo/muy bajo. Sin metodo de aleatorizacion, ocultamiento de asignacion, cegamiento de cuidadores o evaluadores, ni manejo de datos incompletos descritos explicitamente; el reporte de resultados parece completo (area de herida, histologia, CD31/VEGF) sin senales de reporte selectivo.</t>
+          <t>Murine model of S. aureus-infected wounds (female BALB/c, 4 groups: PBS, NIR, NPs, NPs+NIR). The text states "6 mice... were divided into four groups" — an ambiguous and very low per-group animal count. No randomization method, allocation concealment, or blinding of caregivers/assessors is described, and incomplete-data handling is not explicitly addressed; outcome reporting appears complete (wound area, histology, CD31/VEGF) with no sign of selective reporting.</t>
         </is>
       </c>
     </row>
@@ -9394,7 +9394,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Zhao et al., 2022, Journal of Magnesium and Alloys [recuperado en 2da subida]</t>
+          <t>Zhao et al., 2022, Journal of Magnesium and Alloys</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -9538,7 +9538,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Alizadeh &amp; Mahmoodi, 2025, Progress in Biomaterials [recuperado en 2da subida]</t>
+          <t>Alizadeh &amp; Mahmoodi, 2025, Progress in Biomaterials</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">

</xml_diff>